<commit_message>
Update C4 viewer (C5-9)
</commit_message>
<xml_diff>
--- a/c5/downloads/C5/SkyG-Speed-60-BOM.xlsx
+++ b/c5/downloads/C5/SkyG-Speed-60-BOM.xlsx
@@ -2734,7 +2734,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Nylon screw M3 x 12</t>
+          <t>Nylon screw M3 x 8</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
@@ -2745,12 +2745,12 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Nylon PA66 socket or pan head</t>
+          <t>Nylon PA66 pan head</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>M3x12 nylon screw</t>
+          <t>M3x8 nylon screw</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>A 16 mm screw here reaches the aileron servo</t>
+          <t>A 12 mm screw here reaches the aileron servo arm (found with the screws modelled in the assembly)</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>17.2</v>
+        <v>17.3</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>1.89</v>
@@ -4120,7 +4120,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 107.3 g, 15.6 h of printing.</t>
+          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 107.4 g, 15.6 h of printing.</t>
         </is>
       </c>
     </row>

</xml_diff>